<commit_message>
Record the second full run (2026-10-16/17) and its outputs
README: the whole pipeline was run again from the public data on a second
computer (Apple M3, 8 GB RAM) with other versions of some R packages; every
output table was reproduced except the simulated cells of Fig. 1b, whose
counts depend on irlba and RANN. Outputs of that run (figure images, the
Excel workbooks and the Fig. 1 simulation); unused code removed from five
figure scripts (the outputs are unchanged).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/Fig4_Perturbseq/output/SuppTable_random_sets.xlsx
+++ b/figs/Fig4_Perturbseq/output/SuppTable_random_sets.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Random sets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other matching methods" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Random sets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Other matching methods" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -536,7 +536,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Source: figs/Fig4_Perturbseq/output/geneset_random_null.csv (figs/Fig4_Perturbseq/analysis/fig4_random_set_null.py; seed 1) and fig4_other_methods_summary.csv (figs/Fig4_Perturbseq/analysis/fig4_other_methods.py; the same draws); table made by figs/Fig4_Perturbseq/analysis/supp_table_random_sets.py on 2026-10-16.</t>
+          <t>Source: figs/Fig4_Perturbseq/output/geneset_random_null.csv (figs/Fig4_Perturbseq/analysis/fig4_random_set_null.py; seed 1) and fig4_other_methods_summary.csv (figs/Fig4_Perturbseq/analysis/fig4_other_methods.py; the same draws); table made by figs/Fig4_Perturbseq/analysis/supp_table_random_sets.py on 2026-10-17.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fig. 5 with intervals over mice, Supplementary Fig. S5, run times of 1.0.1
Fig. 5, Supplementary Fig. S4 and Supplementary Table 3: the 95% confidence
intervals are obtained by bootstrapping mice (fig5_mice.py and boot_task of
fig5_bench_redo.R), Fig. 5e shows the mean over the tasks of each type
(fig5_task_means.py), the reference-length panel is Fig. 5f, and the panels
are drawn without header lines to fit a 180 x 180 mm page at full size.
Outputs of the run of 2026-10-20.

Supplementary Fig. S5: the interferon-beta response of human peripheral blood
mononuclear cells (analysis/kang, figs/Supp_S5_Kang).

Run time and peak memory measured again with version 1.0.1 of the packages
(Supplementary Table 3, demo/README.md, README.md). The package demos sum the
two rows whose gene names differ only in case (PISD and Pisd) before scoring,
as the packages ask. Outputs of the full run of 2026-10-19.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/Fig4_Perturbseq/output/SuppTable_random_sets.xlsx
+++ b/figs/Fig4_Perturbseq/output/SuppTable_random_sets.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Random sets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Other matching methods" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Random sets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other matching methods" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -536,7 +536,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Source: figs/Fig4_Perturbseq/output/geneset_random_null.csv (figs/Fig4_Perturbseq/analysis/fig4_random_set_null.py; seed 1) and fig4_other_methods_summary.csv (figs/Fig4_Perturbseq/analysis/fig4_other_methods.py; the same draws); table made by figs/Fig4_Perturbseq/analysis/supp_table_random_sets.py on 2026-10-17.</t>
+          <t>Source: figs/Fig4_Perturbseq/output/geneset_random_null.csv (figs/Fig4_Perturbseq/analysis/fig4_random_set_null.py; seed 1) and fig4_other_methods_summary.csv (figs/Fig4_Perturbseq/analysis/fig4_other_methods.py; the same draws); table made by figs/Fig4_Perturbseq/analysis/supp_table_random_sets.py on 2026-10-19.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove the balanced-accuracy analysis; Fig. 4e shows Nr3c1 and Ncoa1 expression in No Stress cells
- Remove fig5_balanced_accuracy.py, its output and the Balanced accuracy sheet of Supplementary Table 3.
- Fig. 4: remove the heatmap of positions (old 4e); the new 4e (fig4e_expression_vs_score.py) sets the expression of
  Nr3c1 and Ncoa1 in the No Stress cells of De Donno et al. against the RFind score of their knock-outs.
- Update Source Data, Supplementary Table 2, run scripts and README accordingly.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/Fig4_Perturbseq/output/SuppTable_random_sets.xlsx
+++ b/figs/Fig4_Perturbseq/output/SuppTable_random_sets.xlsx
@@ -505,7 +505,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>&lt;gene&gt;: % from the opposed end — position of the knock-out counted from the knock-out most opposed to the stress response (1), as a percentage of the knock-outs ranked (as in Fig. 4e; below 50, the opposed side).</t>
+          <t>&lt;gene&gt;: % from the opposed end — position of the knock-out counted from the knock-out most opposed to the stress response (1), as a percentage of the knock-outs ranked (below 50, the opposed side).</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Source: figs/Fig4_Perturbseq/output/geneset_random_null.csv (figs/Fig4_Perturbseq/analysis/fig4_random_set_null.py; seed 1) and fig4_other_methods_summary.csv (figs/Fig4_Perturbseq/analysis/fig4_other_methods.py; the same draws); table made by figs/Fig4_Perturbseq/analysis/supp_table_random_sets.py on 2026-10-19.</t>
+          <t>Source: figs/Fig4_Perturbseq/output/geneset_random_null.csv (figs/Fig4_Perturbseq/analysis/fig4_random_set_null.py; seed 1) and fig4_other_methods_summary.csv (figs/Fig4_Perturbseq/analysis/fig4_other_methods.py; the same draws); table made by figs/Fig4_Perturbseq/analysis/supp_table_random_sets.py on 2026-10-21.</t>
         </is>
       </c>
     </row>

</xml_diff>